<commit_message>
Update refresher excel with todays work
</commit_message>
<xml_diff>
--- a/technical_fluency_project_refresher.xlsx
+++ b/technical_fluency_project_refresher.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saver\01_PROJECT\refresher-dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18862AE8-1031-4B62-BC15-58FF1CF5A394}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D72FF250-0D6E-4ADF-B498-6C8A2AB58DDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Daily plan" sheetId="1" state="hidden" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2578" uniqueCount="1079">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2584" uniqueCount="1084">
   <si>
     <t>Sebastian's October 2026 re-entry plan</t>
   </si>
@@ -3271,13 +3271,28 @@
     <t>In progress</t>
   </si>
   <si>
-    <t xml:space="preserve">First step, find an interesting dataset, that dataset being a speed dating dataset (Data exploration) </t>
-  </si>
-  <si>
     <t>data_explore.ipynb</t>
   </si>
   <si>
     <t>Thinking about ingestion and overall how the data is going to move</t>
+  </si>
+  <si>
+    <t>Skipped</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First step, find an interesting dataset, that dataset being a test taking dataset (Data exploration) </t>
+  </si>
+  <si>
+    <t>Import data set as raw_spf_df using pandas data_profiling tool</t>
+  </si>
+  <si>
+    <t>Look at anomlies within the dataset</t>
+  </si>
+  <si>
+    <t>Use python fuction to make this process easier</t>
+  </si>
+  <si>
+    <t>Ordinal and nominal categories.</t>
   </si>
 </sst>
 </file>
@@ -3837,7 +3852,7 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>0.125</c:v>
+                  <c:v>0.3</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -7243,11 +7258,11 @@
       </c>
       <c r="E11" s="32">
         <f>COUNTIFS('Project Checklist'!$C$3:$C$146,A11,'Project Checklist'!$H$3:$H$146,"Done")</f>
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="F11" s="33">
         <f>IFERROR(E11/D11,0)</f>
-        <v>0.125</v>
+        <v>0.3</v>
       </c>
       <c r="G11" s="32"/>
       <c r="H11" s="32"/>
@@ -7399,7 +7414,7 @@
       </c>
       <c r="B18" s="32">
         <f>COUNTIF('Project Checklist'!H3:H146,"Done")</f>
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C18" s="32"/>
       <c r="D18" s="32"/>
@@ -7420,7 +7435,7 @@
       </c>
       <c r="B19" s="36">
         <f>SUM('Daily Journal'!L3:L38)/60</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C19" s="32"/>
       <c r="D19" s="32"/>
@@ -7441,7 +7456,7 @@
       </c>
       <c r="B20" s="32">
         <f>COUNTIF('Daily Journal'!L3:L38,"&gt;0")</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C20" s="32"/>
       <c r="D20" s="32"/>
@@ -7996,7 +8011,7 @@
         <v>437</v>
       </c>
       <c r="H8" s="32" t="s">
-        <v>1075</v>
+        <v>306</v>
       </c>
       <c r="I8" s="32" t="s">
         <v>445</v>
@@ -8037,7 +8052,7 @@
         <v>439</v>
       </c>
       <c r="H9" s="32" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="I9" s="32" t="s">
         <v>445</v>
@@ -8078,7 +8093,7 @@
         <v>441</v>
       </c>
       <c r="H10" s="32" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="I10" s="32" t="s">
         <v>445</v>
@@ -8119,7 +8134,7 @@
         <v>430</v>
       </c>
       <c r="H11" s="32" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="I11" s="32" t="s">
         <v>456</v>
@@ -8160,7 +8175,7 @@
         <v>437</v>
       </c>
       <c r="H12" s="32" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="I12" s="32" t="s">
         <v>456</v>
@@ -8201,7 +8216,7 @@
         <v>439</v>
       </c>
       <c r="H13" s="32" t="s">
-        <v>311</v>
+        <v>1075</v>
       </c>
       <c r="I13" s="32" t="s">
         <v>456</v>
@@ -8242,7 +8257,7 @@
         <v>441</v>
       </c>
       <c r="H14" s="32" t="s">
-        <v>311</v>
+        <v>1078</v>
       </c>
       <c r="I14" s="32" t="s">
         <v>456</v>
@@ -8283,7 +8298,7 @@
         <v>430</v>
       </c>
       <c r="H15" s="32" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="I15" s="32" t="s">
         <v>467</v>
@@ -8324,7 +8339,7 @@
         <v>437</v>
       </c>
       <c r="H16" s="32" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="I16" s="32" t="s">
         <v>467</v>
@@ -13792,10 +13807,10 @@
         <v>1</v>
       </c>
       <c r="F3" s="32" t="s">
-        <v>1076</v>
+        <v>1079</v>
       </c>
       <c r="G3" s="32" t="s">
-        <v>1078</v>
+        <v>1077</v>
       </c>
       <c r="H3" s="32"/>
       <c r="I3" s="32"/>
@@ -13805,7 +13820,7 @@
         <v>120</v>
       </c>
       <c r="M3" s="32" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="27.6">
@@ -13823,16 +13838,22 @@
       </c>
       <c r="E4" s="33">
         <f>IFERROR(COUNTIFS('Project Checklist'!$A$3:$A$146,A4,'Project Checklist'!$H$3:$H$146,"Done")/COUNTIF('Project Checklist'!$A$3:$A$146,A4),0)</f>
-        <v>0.25</v>
-      </c>
-      <c r="F4" s="32"/>
+        <v>1</v>
+      </c>
+      <c r="F4" s="32" t="s">
+        <v>1080</v>
+      </c>
       <c r="G4" s="32"/>
       <c r="H4" s="32"/>
       <c r="I4" s="32"/>
       <c r="J4" s="32"/>
       <c r="K4" s="32"/>
-      <c r="L4" s="34"/>
-      <c r="M4" s="32"/>
+      <c r="L4" s="34">
+        <v>30</v>
+      </c>
+      <c r="M4" s="32" t="s">
+        <v>1076</v>
+      </c>
     </row>
     <row r="5" spans="1:13" ht="27.6">
       <c r="A5" s="31">
@@ -13849,16 +13870,26 @@
       </c>
       <c r="E5" s="33">
         <f>IFERROR(COUNTIFS('Project Checklist'!$A$3:$A$146,A5,'Project Checklist'!$H$3:$H$146,"Done")/COUNTIF('Project Checklist'!$A$3:$A$146,A5),0)</f>
-        <v>0</v>
-      </c>
-      <c r="F5" s="32"/>
-      <c r="G5" s="32"/>
-      <c r="H5" s="32"/>
+        <v>0.5</v>
+      </c>
+      <c r="F5" s="32" t="s">
+        <v>1081</v>
+      </c>
+      <c r="G5" s="32" t="s">
+        <v>1082</v>
+      </c>
+      <c r="H5" s="32" t="s">
+        <v>1083</v>
+      </c>
       <c r="I5" s="32"/>
       <c r="J5" s="32"/>
       <c r="K5" s="32"/>
-      <c r="L5" s="34"/>
-      <c r="M5" s="32"/>
+      <c r="L5" s="34">
+        <v>30</v>
+      </c>
+      <c r="M5" s="32" t="s">
+        <v>1076</v>
+      </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="31">
@@ -13875,7 +13906,7 @@
       </c>
       <c r="E6" s="33">
         <f>IFERROR(COUNTIFS('Project Checklist'!$A$3:$A$146,A6,'Project Checklist'!$H$3:$H$146,"Done")/COUNTIF('Project Checklist'!$A$3:$A$146,A6),0)</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F6" s="32"/>
       <c r="G6" s="32"/>

</xml_diff>

<commit_message>
Begin work on descriptive analysis
</commit_message>
<xml_diff>
--- a/technical_fluency_project_refresher.xlsx
+++ b/technical_fluency_project_refresher.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saver\01_PROJECT\refresher-dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D72FF250-0D6E-4ADF-B498-6C8A2AB58DDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D85394A0-C234-46A0-8E4B-4D906E8973A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2584" uniqueCount="1084">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2587" uniqueCount="1087">
   <si>
     <t>Sebastian's October 2026 re-entry plan</t>
   </si>
@@ -3293,6 +3293,17 @@
   </si>
   <si>
     <t>Ordinal and nominal categories.</t>
+  </si>
+  <si>
+    <t>Grain became much clearer when I related it to organizational levels such as wing, squadron, flight, and individual records. I also reinforced that cleaning should be based on the analytical purpose rather than making changes simply because a cleaning technique exists. I removed 293 records whose missing information prevented them from contributing meaningfully to the planned analysis and otherwise preserved the dataset because it was already relatively clean.</t>
+  </si>
+  <si>
+    <t>Numerator   = total students
+Denominator = number of classrooms
+Metric      = average students per classroom</t>
+  </si>
+  <si>
+    <t>Working with establishing the numerator, denominator, and metric as well as the exclusion</t>
   </si>
 </sst>
 </file>
@@ -3601,11 +3612,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -3616,9 +3625,11 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3852,7 +3863,7 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>0.3</c:v>
+                  <c:v>0.42499999999999999</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -7258,11 +7269,11 @@
       </c>
       <c r="E11" s="32">
         <f>COUNTIFS('Project Checklist'!$C$3:$C$146,A11,'Project Checklist'!$H$3:$H$146,"Done")</f>
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F11" s="33">
         <f>IFERROR(E11/D11,0)</f>
-        <v>0.3</v>
+        <v>0.42499999999999999</v>
       </c>
       <c r="G11" s="32"/>
       <c r="H11" s="32"/>
@@ -7414,7 +7425,7 @@
       </c>
       <c r="B18" s="32">
         <f>COUNTIF('Project Checklist'!H3:H146,"Done")</f>
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C18" s="32"/>
       <c r="D18" s="32"/>
@@ -7435,7 +7446,7 @@
       </c>
       <c r="B19" s="36">
         <f>SUM('Daily Journal'!L3:L38)/60</f>
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="C19" s="32"/>
       <c r="D19" s="32"/>
@@ -7456,7 +7467,7 @@
       </c>
       <c r="B20" s="32">
         <f>COUNTIF('Daily Journal'!L3:L38,"&gt;0")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C20" s="32"/>
       <c r="D20" s="32"/>
@@ -7726,21 +7737,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="24" customHeight="1">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="42" t="s">
         <v>415</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
-      <c r="H1" s="38"/>
-      <c r="I1" s="38"/>
-      <c r="J1" s="38"/>
-      <c r="K1" s="38"/>
-      <c r="L1" s="38"/>
-      <c r="M1" s="38"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+      <c r="K1" s="43"/>
+      <c r="L1" s="43"/>
+      <c r="M1" s="43"/>
     </row>
     <row r="2" spans="1:13">
       <c r="A2" s="30" t="s">
@@ -8216,7 +8227,7 @@
         <v>439</v>
       </c>
       <c r="H13" s="32" t="s">
-        <v>1075</v>
+        <v>306</v>
       </c>
       <c r="I13" s="32" t="s">
         <v>456</v>
@@ -8380,7 +8391,7 @@
         <v>439</v>
       </c>
       <c r="H17" s="32" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="I17" s="32" t="s">
         <v>467</v>
@@ -8421,7 +8432,7 @@
         <v>441</v>
       </c>
       <c r="H18" s="32" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="I18" s="32" t="s">
         <v>467</v>
@@ -8462,7 +8473,7 @@
         <v>430</v>
       </c>
       <c r="H19" s="32" t="s">
-        <v>311</v>
+        <v>1075</v>
       </c>
       <c r="I19" s="32" t="s">
         <v>478</v>
@@ -8503,7 +8514,7 @@
         <v>437</v>
       </c>
       <c r="H20" s="32" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="I20" s="32" t="s">
         <v>478</v>
@@ -8585,7 +8596,7 @@
         <v>441</v>
       </c>
       <c r="H22" s="32" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="I22" s="32" t="s">
         <v>478</v>
@@ -13708,8 +13719,9 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -13732,21 +13744,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="24" customHeight="1">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="37" t="s">
         <v>825</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="43"/>
-      <c r="I1" s="43"/>
-      <c r="J1" s="43"/>
-      <c r="K1" s="43"/>
-      <c r="L1" s="43"/>
-      <c r="M1" s="43"/>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
+      <c r="E1" s="38"/>
+      <c r="F1" s="38"/>
+      <c r="G1" s="38"/>
+      <c r="H1" s="38"/>
+      <c r="I1" s="38"/>
+      <c r="J1" s="38"/>
+      <c r="K1" s="38"/>
+      <c r="L1" s="38"/>
+      <c r="M1" s="38"/>
     </row>
     <row r="2" spans="1:13" ht="27.6">
       <c r="A2" s="30" t="s">
@@ -13870,7 +13882,7 @@
       </c>
       <c r="E5" s="33">
         <f>IFERROR(COUNTIFS('Project Checklist'!$A$3:$A$146,A5,'Project Checklist'!$H$3:$H$146,"Done")/COUNTIF('Project Checklist'!$A$3:$A$146,A5),0)</f>
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="F5" s="32" t="s">
         <v>1081</v>
@@ -13891,7 +13903,7 @@
         <v>1076</v>
       </c>
     </row>
-    <row r="6" spans="1:13">
+    <row r="6" spans="1:13" ht="151.80000000000001">
       <c r="A6" s="31">
         <v>46324</v>
       </c>
@@ -13906,18 +13918,22 @@
       </c>
       <c r="E6" s="33">
         <f>IFERROR(COUNTIFS('Project Checklist'!$A$3:$A$146,A6,'Project Checklist'!$H$3:$H$146,"Done")/COUNTIF('Project Checklist'!$A$3:$A$146,A6),0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F6" s="32"/>
       <c r="G6" s="32"/>
-      <c r="H6" s="32"/>
+      <c r="H6" s="32" t="s">
+        <v>1084</v>
+      </c>
       <c r="I6" s="32"/>
       <c r="J6" s="32"/>
       <c r="K6" s="32"/>
-      <c r="L6" s="34"/>
+      <c r="L6" s="34">
+        <v>30</v>
+      </c>
       <c r="M6" s="32"/>
     </row>
-    <row r="7" spans="1:13" ht="27.6">
+    <row r="7" spans="1:13" ht="41.4">
       <c r="A7" s="31">
         <v>46325</v>
       </c>
@@ -13932,11 +13948,15 @@
       </c>
       <c r="E7" s="33">
         <f>IFERROR(COUNTIFS('Project Checklist'!$A$3:$A$146,A7,'Project Checklist'!$H$3:$H$146,"Done")/COUNTIF('Project Checklist'!$A$3:$A$146,A7),0)</f>
-        <v>0</v>
-      </c>
-      <c r="F7" s="32"/>
+        <v>0.5</v>
+      </c>
+      <c r="F7" s="32" t="s">
+        <v>1086</v>
+      </c>
       <c r="G7" s="32"/>
-      <c r="H7" s="32"/>
+      <c r="H7" s="32" t="s">
+        <v>1085</v>
+      </c>
       <c r="I7" s="32"/>
       <c r="J7" s="32"/>
       <c r="K7" s="32"/>
@@ -14812,14 +14832,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="24" customHeight="1">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="37" t="s">
         <v>835</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
+      <c r="E1" s="38"/>
+      <c r="F1" s="38"/>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="30" t="s">
@@ -15443,13 +15463,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="24" customHeight="1">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="37" t="s">
         <v>981</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
+      <c r="E1" s="38"/>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="30" t="s">
@@ -15710,10 +15730,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="24" customHeight="1">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="37" t="s">
         <v>1049</v>
       </c>
-      <c r="B1" s="43"/>
+      <c r="B1" s="38"/>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="30" t="s">

</xml_diff>

<commit_message>
Continue to work through EDA
</commit_message>
<xml_diff>
--- a/technical_fluency_project_refresher.xlsx
+++ b/technical_fluency_project_refresher.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saver\01_PROJECT\refresher-dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D85394A0-C234-46A0-8E4B-4D906E8973A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{108C8AE4-7C17-49CC-995D-C067F4F01184}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Daily plan" sheetId="1" state="hidden" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2587" uniqueCount="1087">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2587" uniqueCount="1086">
   <si>
     <t>Sebastian's October 2026 re-entry plan</t>
   </si>
@@ -3266,9 +3266,6 @@
   </si>
   <si>
     <t>The original Daily plan, Progress, and Guide remain in the workbook as the warm-up/history from the first phase.</t>
-  </si>
-  <si>
-    <t>In progress</t>
   </si>
   <si>
     <t>data_explore.ipynb</t>
@@ -3863,7 +3860,7 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>0.42499999999999999</c:v>
+                  <c:v>0.55000000000000004</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -7269,11 +7266,11 @@
       </c>
       <c r="E11" s="32">
         <f>COUNTIFS('Project Checklist'!$C$3:$C$146,A11,'Project Checklist'!$H$3:$H$146,"Done")</f>
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F11" s="33">
         <f>IFERROR(E11/D11,0)</f>
-        <v>0.42499999999999999</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="G11" s="32"/>
       <c r="H11" s="32"/>
@@ -7425,7 +7422,7 @@
       </c>
       <c r="B18" s="32">
         <f>COUNTIF('Project Checklist'!H3:H146,"Done")</f>
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C18" s="32"/>
       <c r="D18" s="32"/>
@@ -8268,7 +8265,7 @@
         <v>441</v>
       </c>
       <c r="H14" s="32" t="s">
-        <v>1078</v>
+        <v>1077</v>
       </c>
       <c r="I14" s="32" t="s">
         <v>456</v>
@@ -8473,7 +8470,7 @@
         <v>430</v>
       </c>
       <c r="H19" s="32" t="s">
-        <v>1075</v>
+        <v>306</v>
       </c>
       <c r="I19" s="32" t="s">
         <v>478</v>
@@ -8555,7 +8552,7 @@
         <v>439</v>
       </c>
       <c r="H21" s="32" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="I21" s="32" t="s">
         <v>478</v>
@@ -8637,7 +8634,7 @@
         <v>430</v>
       </c>
       <c r="H23" s="32" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="I23" s="32" t="s">
         <v>489</v>
@@ -8678,7 +8675,7 @@
         <v>437</v>
       </c>
       <c r="H24" s="32" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="I24" s="32" t="s">
         <v>489</v>
@@ -8719,7 +8716,7 @@
         <v>439</v>
       </c>
       <c r="H25" s="32" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="I25" s="32" t="s">
         <v>489</v>
@@ -13819,10 +13816,10 @@
         <v>1</v>
       </c>
       <c r="F3" s="32" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
       <c r="G3" s="32" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="H3" s="32"/>
       <c r="I3" s="32"/>
@@ -13832,7 +13829,7 @@
         <v>120</v>
       </c>
       <c r="M3" s="32" t="s">
-        <v>1076</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="27.6">
@@ -13853,7 +13850,7 @@
         <v>1</v>
       </c>
       <c r="F4" s="32" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
       <c r="G4" s="32"/>
       <c r="H4" s="32"/>
@@ -13864,7 +13861,7 @@
         <v>30</v>
       </c>
       <c r="M4" s="32" t="s">
-        <v>1076</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="27.6">
@@ -13885,13 +13882,13 @@
         <v>0.75</v>
       </c>
       <c r="F5" s="32" t="s">
+        <v>1080</v>
+      </c>
+      <c r="G5" s="32" t="s">
         <v>1081</v>
       </c>
-      <c r="G5" s="32" t="s">
+      <c r="H5" s="32" t="s">
         <v>1082</v>
-      </c>
-      <c r="H5" s="32" t="s">
-        <v>1083</v>
       </c>
       <c r="I5" s="32"/>
       <c r="J5" s="32"/>
@@ -13900,7 +13897,7 @@
         <v>30</v>
       </c>
       <c r="M5" s="32" t="s">
-        <v>1076</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="151.80000000000001">
@@ -13923,7 +13920,7 @@
       <c r="F6" s="32"/>
       <c r="G6" s="32"/>
       <c r="H6" s="32" t="s">
-        <v>1084</v>
+        <v>1083</v>
       </c>
       <c r="I6" s="32"/>
       <c r="J6" s="32"/>
@@ -13948,14 +13945,14 @@
       </c>
       <c r="E7" s="33">
         <f>IFERROR(COUNTIFS('Project Checklist'!$A$3:$A$146,A7,'Project Checklist'!$H$3:$H$146,"Done")/COUNTIF('Project Checklist'!$A$3:$A$146,A7),0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F7" s="32" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="G7" s="32"/>
       <c r="H7" s="32" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
       <c r="I7" s="32"/>
       <c r="J7" s="32"/>
@@ -13978,7 +13975,7 @@
       </c>
       <c r="E8" s="33">
         <f>IFERROR(COUNTIFS('Project Checklist'!$A$3:$A$146,A8,'Project Checklist'!$H$3:$H$146,"Done")/COUNTIF('Project Checklist'!$A$3:$A$146,A8),0)</f>
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="F8" s="32"/>
       <c r="G8" s="32"/>

</xml_diff>